<commit_message>
Corregir nombre del integrante: Camilo Bastidas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SGxJnM4mGNnRkmsMPkg1Yf
</commit_message>
<xml_diff>
--- a/descargas/Product_Backlog_MatchPoint.xlsx
+++ b/descargas/Product_Backlog_MatchPoint.xlsx
@@ -1669,7 +1669,7 @@
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>EQUIPO PROPUESTO: Santiago Solano · Scrum Master  |  Maicol Rubiano · Backend Developer  |  Diego Romero · Frontend Developer  |  Camilo Bastias · Database Administrator (DBA)</t>
+          <t>EQUIPO PROPUESTO: Santiago Solano · Scrum Master  |  Maicol Rubiano · Backend Developer  |  Diego Romero · Frontend Developer  |  Camilo Bastidas · Database Administrator (DBA)</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="K11" s="26" t="inlineStr">
         <is>
-          <t>Camilo Bastias · Database Administrator (DBA)</t>
+          <t>Camilo Bastidas · Database Administrator (DBA)</t>
         </is>
       </c>
       <c r="L11" s="26" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="K15" s="26" t="inlineStr">
         <is>
-          <t>Camilo Bastias · Database Administrator (DBA)</t>
+          <t>Camilo Bastidas · Database Administrator (DBA)</t>
         </is>
       </c>
       <c r="L15" s="26" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="K22" s="30" t="inlineStr">
         <is>
-          <t>Camilo Bastias · Database Administrator (DBA)</t>
+          <t>Camilo Bastidas · Database Administrator (DBA)</t>
         </is>
       </c>
       <c r="L22" s="30" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="K23" s="26" t="inlineStr">
         <is>
-          <t>Camilo Bastias · Database Administrator (DBA)</t>
+          <t>Camilo Bastidas · Database Administrator (DBA)</t>
         </is>
       </c>
       <c r="L23" s="26" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="K24" s="30" t="inlineStr">
         <is>
-          <t>Camilo Bastias · Database Administrator (DBA)</t>
+          <t>Camilo Bastidas · Database Administrator (DBA)</t>
         </is>
       </c>
       <c r="L24" s="30" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="K25" s="26" t="inlineStr">
         <is>
-          <t>Camilo Bastias · Database Administrator (DBA)</t>
+          <t>Camilo Bastidas · Database Administrator (DBA)</t>
         </is>
       </c>
       <c r="L25" s="26" t="inlineStr">

</xml_diff>